<commit_message>
Se implmento a la base de datos
</commit_message>
<xml_diff>
--- a/SistemaInventario/Inventario_Reporte.xlsx
+++ b/SistemaInventario/Inventario_Reporte.xlsx
@@ -26,16 +26,16 @@
     <t>Precio</t>
   </si>
   <si>
-    <t>1780764720437</t>
+    <t>1780772464670</t>
   </si>
   <si>
-    <t>Lap Top</t>
+    <t>ddfdf</t>
   </si>
   <si>
-    <t>1780764834115</t>
+    <t>1780772507320</t>
   </si>
   <si>
-    <t xml:space="preserve">Proyector </t>
+    <t>LapTop</t>
   </si>
 </sst>
 </file>
@@ -105,10 +105,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>20.0</v>
+        <v>12.0</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>1850.0</v>
+        <v>1500.0</v>
       </c>
     </row>
     <row r="3">
@@ -119,10 +119,10 @@
         <v>7</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>1500.0</v>
+        <v>1850.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se agrego el login, menú principal
</commit_message>
<xml_diff>
--- a/SistemaInventario/Inventario_Reporte.xlsx
+++ b/SistemaInventario/Inventario_Reporte.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>ID</t>
   </si>
@@ -36,6 +36,12 @@
   </si>
   <si>
     <t>LapTop</t>
+  </si>
+  <si>
+    <t>1780781891253</t>
+  </si>
+  <si>
+    <t>Proyector</t>
   </si>
 </sst>
 </file>
@@ -80,7 +86,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -125,6 +131,20 @@
         <v>1850.0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C4" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="D4" t="n" s="0">
+        <v>1600.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>